<commit_message>
add: fluxo completo funcionando
</commit_message>
<xml_diff>
--- a/dataset/Request-Urllib.xlsx
+++ b/dataset/Request-Urllib.xlsx
@@ -1,12 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Request-Urllib" sheetId="1" r:id="rId5"/>
+    <sheet r:id="rId1" sheetId="1" name="Request-Urllib"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -4808,22 +4811,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <color rgb="FF0000ff"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4831,50 +4840,62 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="4">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -4901,22 +4922,82 @@
         <a:srgbClr val="46BDC6"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155CC"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -4928,146 +5009,186 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:tint val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="9500"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot rev="0" lon="0" lat="0"/>
+            </a:camera>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:tint val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H201"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="3" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="3" width="13.005" customWidth="1" bestFit="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5093,7 +5214,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -5119,7 +5240,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -5145,7 +5266,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -5171,7 +5292,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -5197,7 +5318,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
       <c r="A6" s="1" t="s">
         <v>31</v>
       </c>
@@ -5223,7 +5344,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
       <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
@@ -5249,7 +5370,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
       <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
@@ -5275,7 +5396,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
       <c r="A9" s="1" t="s">
         <v>41</v>
       </c>
@@ -5301,7 +5422,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
       <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
@@ -5327,7 +5448,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -5353,7 +5474,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
       <c r="A12" s="1" t="s">
         <v>41</v>
       </c>
@@ -5379,7 +5500,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
       <c r="A13" s="1" t="s">
         <v>41</v>
       </c>
@@ -5405,7 +5526,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
       <c r="A14" s="1" t="s">
         <v>54</v>
       </c>
@@ -5431,7 +5552,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
       <c r="A15" s="1" t="s">
         <v>54</v>
       </c>
@@ -5457,7 +5578,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -5483,7 +5604,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
       <c r="A17" s="1" t="s">
         <v>63</v>
       </c>
@@ -5509,7 +5630,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
       <c r="A18" s="1" t="s">
         <v>63</v>
       </c>
@@ -5535,7 +5656,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
       <c r="A19" s="1" t="s">
         <v>63</v>
       </c>
@@ -5561,7 +5682,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
       <c r="A20" s="1" t="s">
         <v>63</v>
       </c>
@@ -5587,7 +5708,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
       <c r="A21" s="1" t="s">
         <v>63</v>
       </c>
@@ -5613,7 +5734,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18">
       <c r="A22" s="1" t="s">
         <v>76</v>
       </c>
@@ -5639,7 +5760,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="23">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18">
       <c r="A23" s="1" t="s">
         <v>81</v>
       </c>
@@ -5665,7 +5786,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18">
       <c r="A24" s="1" t="s">
         <v>86</v>
       </c>
@@ -5691,7 +5812,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18">
       <c r="A25" s="1" t="s">
         <v>91</v>
       </c>
@@ -5717,7 +5838,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="26">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18">
       <c r="A26" s="1" t="s">
         <v>96</v>
       </c>
@@ -5743,7 +5864,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18">
       <c r="A27" s="1" t="s">
         <v>96</v>
       </c>
@@ -5769,7 +5890,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="28">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18">
       <c r="A28" s="1" t="s">
         <v>103</v>
       </c>
@@ -5795,7 +5916,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="29">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18">
       <c r="A29" s="1" t="s">
         <v>103</v>
       </c>
@@ -5821,7 +5942,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="30">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
       <c r="A30" s="1" t="s">
         <v>111</v>
       </c>
@@ -5847,7 +5968,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
       <c r="A31" s="1" t="s">
         <v>111</v>
       </c>
@@ -5873,7 +5994,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="32">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
       <c r="A32" s="1" t="s">
         <v>111</v>
       </c>
@@ -5899,7 +6020,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
       <c r="A33" s="1" t="s">
         <v>111</v>
       </c>
@@ -5925,7 +6046,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="34">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18">
       <c r="A34" s="1" t="s">
         <v>111</v>
       </c>
@@ -5951,7 +6072,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="35">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18">
       <c r="A35" s="1" t="s">
         <v>111</v>
       </c>
@@ -5977,7 +6098,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="36">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18">
       <c r="A36" s="1" t="s">
         <v>111</v>
       </c>
@@ -6003,7 +6124,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18">
       <c r="A37" s="1" t="s">
         <v>130</v>
       </c>
@@ -6029,7 +6150,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="38">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18">
       <c r="A38" s="1" t="s">
         <v>130</v>
       </c>
@@ -6055,7 +6176,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="39">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18">
       <c r="A39" s="1" t="s">
         <v>130</v>
       </c>
@@ -6081,7 +6202,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="40">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18">
       <c r="A40" s="1" t="s">
         <v>140</v>
       </c>
@@ -6107,7 +6228,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18">
       <c r="A41" s="1" t="s">
         <v>140</v>
       </c>
@@ -6133,7 +6254,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="42">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18">
       <c r="A42" s="1" t="s">
         <v>147</v>
       </c>
@@ -6159,7 +6280,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="43">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18">
       <c r="A43" s="1" t="s">
         <v>152</v>
       </c>
@@ -6185,7 +6306,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="44">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18">
       <c r="A44" s="1" t="s">
         <v>152</v>
       </c>
@@ -6211,7 +6332,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="45">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18">
       <c r="A45" s="1" t="s">
         <v>159</v>
       </c>
@@ -6237,7 +6358,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="46">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18">
       <c r="A46" s="1" t="s">
         <v>164</v>
       </c>
@@ -6263,7 +6384,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="47">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18">
       <c r="A47" s="1" t="s">
         <v>164</v>
       </c>
@@ -6289,7 +6410,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="48">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18">
       <c r="A48" s="1" t="s">
         <v>171</v>
       </c>
@@ -6315,7 +6436,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="49">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18">
       <c r="A49" s="1" t="s">
         <v>171</v>
       </c>
@@ -6341,7 +6462,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="50">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18">
       <c r="A50" s="1" t="s">
         <v>178</v>
       </c>
@@ -6367,7 +6488,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="51">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18">
       <c r="A51" s="1" t="s">
         <v>178</v>
       </c>
@@ -6393,7 +6514,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="52">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18">
       <c r="A52" s="1" t="s">
         <v>178</v>
       </c>
@@ -6419,7 +6540,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18">
       <c r="A53" s="1" t="s">
         <v>178</v>
       </c>
@@ -6445,7 +6566,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="54">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18">
       <c r="A54" s="1" t="s">
         <v>191</v>
       </c>
@@ -6471,7 +6592,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="55">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18">
       <c r="A55" s="1" t="s">
         <v>191</v>
       </c>
@@ -6497,7 +6618,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="56">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18">
       <c r="A56" s="1" t="s">
         <v>191</v>
       </c>
@@ -6523,7 +6644,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="57">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="78">
       <c r="A57" s="1" t="s">
         <v>201</v>
       </c>
@@ -6549,7 +6670,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="58">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="78">
       <c r="A58" s="1" t="s">
         <v>201</v>
       </c>
@@ -6575,7 +6696,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="59">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="30">
       <c r="A59" s="1" t="s">
         <v>201</v>
       </c>
@@ -6601,7 +6722,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="60">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="66">
       <c r="A60" s="1" t="s">
         <v>201</v>
       </c>
@@ -6627,7 +6748,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="61">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="54">
       <c r="A61" s="1" t="s">
         <v>212</v>
       </c>
@@ -6653,7 +6774,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="62">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="246">
       <c r="A62" s="1" t="s">
         <v>212</v>
       </c>
@@ -6679,7 +6800,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="63">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18">
       <c r="A63" s="1" t="s">
         <v>212</v>
       </c>
@@ -6705,7 +6826,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="64">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="258">
       <c r="A64" s="1" t="s">
         <v>221</v>
       </c>
@@ -6731,7 +6852,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="65">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="246">
       <c r="A65" s="1" t="s">
         <v>221</v>
       </c>
@@ -6757,7 +6878,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="66">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="66">
       <c r="A66" s="1" t="s">
         <v>228</v>
       </c>
@@ -6783,7 +6904,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="67">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18">
       <c r="A67" s="1" t="s">
         <v>228</v>
       </c>
@@ -6809,7 +6930,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="68">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="462">
       <c r="A68" s="1" t="s">
         <v>235</v>
       </c>
@@ -6835,7 +6956,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="69">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18">
       <c r="A69" s="1" t="s">
         <v>240</v>
       </c>
@@ -6861,7 +6982,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="70">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="726">
       <c r="A70" s="1" t="s">
         <v>245</v>
       </c>
@@ -6887,7 +7008,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="71">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="54">
       <c r="A71" s="1" t="s">
         <v>250</v>
       </c>
@@ -6913,7 +7034,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="72">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="54">
       <c r="A72" s="1" t="s">
         <v>250</v>
       </c>
@@ -6939,7 +7060,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="73">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="138">
       <c r="A73" s="1" t="s">
         <v>250</v>
       </c>
@@ -6965,7 +7086,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="74">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18">
       <c r="A74" s="1" t="s">
         <v>250</v>
       </c>
@@ -6991,7 +7112,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="75">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18">
       <c r="A75" s="1" t="s">
         <v>250</v>
       </c>
@@ -7017,7 +7138,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="76">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18">
       <c r="A76" s="1" t="s">
         <v>250</v>
       </c>
@@ -7043,7 +7164,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="77">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18">
       <c r="A77" s="1" t="s">
         <v>250</v>
       </c>
@@ -7069,7 +7190,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="78">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18">
       <c r="A78" s="1" t="s">
         <v>250</v>
       </c>
@@ -7095,7 +7216,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="79">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18">
       <c r="A79" s="1" t="s">
         <v>250</v>
       </c>
@@ -7121,7 +7242,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="80">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18">
       <c r="A80" s="1" t="s">
         <v>250</v>
       </c>
@@ -7147,7 +7268,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="81">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18">
       <c r="A81" s="1" t="s">
         <v>250</v>
       </c>
@@ -7173,7 +7294,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="82">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18">
       <c r="A82" s="1" t="s">
         <v>250</v>
       </c>
@@ -7199,7 +7320,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="83">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18">
       <c r="A83" s="1" t="s">
         <v>250</v>
       </c>
@@ -7225,7 +7346,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="84">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18">
       <c r="A84" s="1" t="s">
         <v>250</v>
       </c>
@@ -7251,7 +7372,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="85">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18">
       <c r="A85" s="1" t="s">
         <v>250</v>
       </c>
@@ -7277,7 +7398,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="86">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18">
       <c r="A86" s="1" t="s">
         <v>250</v>
       </c>
@@ -7303,7 +7424,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="87">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18">
       <c r="A87" s="1" t="s">
         <v>250</v>
       </c>
@@ -7329,7 +7450,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="88">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18">
       <c r="A88" s="1" t="s">
         <v>250</v>
       </c>
@@ -7355,7 +7476,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="89">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18">
       <c r="A89" s="1" t="s">
         <v>250</v>
       </c>
@@ -7381,7 +7502,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="90">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18">
       <c r="A90" s="1" t="s">
         <v>250</v>
       </c>
@@ -7407,7 +7528,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="91">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18">
       <c r="A91" s="1" t="s">
         <v>294</v>
       </c>
@@ -7433,7 +7554,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="92">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18">
       <c r="A92" s="1" t="s">
         <v>299</v>
       </c>
@@ -7459,7 +7580,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="93">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18">
       <c r="A93" s="1" t="s">
         <v>299</v>
       </c>
@@ -7485,7 +7606,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="94">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18">
       <c r="A94" s="1" t="s">
         <v>307</v>
       </c>
@@ -7511,7 +7632,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="95">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18">
       <c r="A95" s="1" t="s">
         <v>312</v>
       </c>
@@ -7537,7 +7658,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="96">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18">
       <c r="A96" s="1" t="s">
         <v>312</v>
       </c>
@@ -7563,7 +7684,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="97">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18">
       <c r="A97" s="1" t="s">
         <v>312</v>
       </c>
@@ -7589,7 +7710,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="98">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18">
       <c r="A98" s="1" t="s">
         <v>322</v>
       </c>
@@ -7615,7 +7736,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="99">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18">
       <c r="A99" s="1" t="s">
         <v>322</v>
       </c>
@@ -7641,7 +7762,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="100">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18">
       <c r="A100" s="1" t="s">
         <v>322</v>
       </c>
@@ -7667,7 +7788,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="101">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18">
       <c r="A101" s="1" t="s">
         <v>333</v>
       </c>
@@ -7693,7 +7814,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="102">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18">
       <c r="A102" s="1" t="s">
         <v>333</v>
       </c>
@@ -7719,7 +7840,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="103">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18">
       <c r="A103" s="1" t="s">
         <v>340</v>
       </c>
@@ -7745,7 +7866,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="104">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18">
       <c r="A104" s="1" t="s">
         <v>345</v>
       </c>
@@ -7771,7 +7892,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="105">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18">
       <c r="A105" s="1" t="s">
         <v>345</v>
       </c>
@@ -7797,7 +7918,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="106">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18">
       <c r="A106" s="1" t="s">
         <v>353</v>
       </c>
@@ -7823,7 +7944,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="107">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18">
       <c r="A107" s="1" t="s">
         <v>353</v>
       </c>
@@ -7849,7 +7970,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="108">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18">
       <c r="A108" s="1" t="s">
         <v>359</v>
       </c>
@@ -7875,7 +7996,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="109">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18">
       <c r="A109" s="1" t="s">
         <v>364</v>
       </c>
@@ -7901,7 +8022,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="110">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18">
       <c r="A110" s="1" t="s">
         <v>364</v>
       </c>
@@ -7927,7 +8048,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="111">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18">
       <c r="A111" s="1" t="s">
         <v>371</v>
       </c>
@@ -7953,7 +8074,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="112">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18">
       <c r="A112" s="1" t="s">
         <v>371</v>
       </c>
@@ -7979,7 +8100,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="113">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18">
       <c r="A113" s="1" t="s">
         <v>371</v>
       </c>
@@ -8005,7 +8126,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="114">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18">
       <c r="A114" s="1" t="s">
         <v>381</v>
       </c>
@@ -8031,7 +8152,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="115">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18">
       <c r="A115" s="1" t="s">
         <v>381</v>
       </c>
@@ -8057,7 +8178,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="116">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18">
       <c r="A116" s="1" t="s">
         <v>381</v>
       </c>
@@ -8083,7 +8204,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="117">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18">
       <c r="A117" s="1" t="s">
         <v>390</v>
       </c>
@@ -8109,7 +8230,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="118">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18">
       <c r="A118" s="1" t="s">
         <v>395</v>
       </c>
@@ -8135,7 +8256,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="119">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18">
       <c r="A119" s="1" t="s">
         <v>395</v>
       </c>
@@ -8161,7 +8282,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="120">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18">
       <c r="A120" s="1" t="s">
         <v>395</v>
       </c>
@@ -8187,7 +8308,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="121">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18">
       <c r="A121" s="1" t="s">
         <v>404</v>
       </c>
@@ -8213,7 +8334,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="122">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18">
       <c r="A122" s="1" t="s">
         <v>409</v>
       </c>
@@ -8239,7 +8360,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="123">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18">
       <c r="A123" s="1" t="s">
         <v>409</v>
       </c>
@@ -8265,7 +8386,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="124">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18">
       <c r="A124" s="1" t="s">
         <v>417</v>
       </c>
@@ -8291,7 +8412,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="125">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18">
       <c r="A125" s="1" t="s">
         <v>417</v>
       </c>
@@ -8317,7 +8438,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="126">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18">
       <c r="A126" s="1" t="s">
         <v>423</v>
       </c>
@@ -8343,7 +8464,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="127">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18">
       <c r="A127" s="1" t="s">
         <v>423</v>
       </c>
@@ -8369,7 +8490,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="128">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18">
       <c r="A128" s="1" t="s">
         <v>429</v>
       </c>
@@ -8395,7 +8516,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="129">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18">
       <c r="A129" s="1" t="s">
         <v>434</v>
       </c>
@@ -8421,7 +8542,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="130">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18">
       <c r="A130" s="1" t="s">
         <v>434</v>
       </c>
@@ -8447,7 +8568,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="131">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18">
       <c r="A131" s="1" t="s">
         <v>434</v>
       </c>
@@ -8473,7 +8594,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="132">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18">
       <c r="A132" s="1" t="s">
         <v>443</v>
       </c>
@@ -8499,7 +8620,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="133">
+    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18">
       <c r="A133" s="1" t="s">
         <v>443</v>
       </c>
@@ -8525,7 +8646,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="134">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18">
       <c r="A134" s="1" t="s">
         <v>450</v>
       </c>
@@ -8551,7 +8672,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="135">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18">
       <c r="A135" s="1" t="s">
         <v>455</v>
       </c>
@@ -8577,7 +8698,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="136">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18">
       <c r="A136" s="1" t="s">
         <v>455</v>
       </c>
@@ -8603,7 +8724,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="137">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18">
       <c r="A137" s="1" t="s">
         <v>455</v>
       </c>
@@ -8629,7 +8750,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="138">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18">
       <c r="A138" s="1" t="s">
         <v>464</v>
       </c>
@@ -8655,7 +8776,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="139">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18">
       <c r="A139" s="1" t="s">
         <v>469</v>
       </c>
@@ -8681,7 +8802,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="140">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18">
       <c r="A140" s="1" t="s">
         <v>469</v>
       </c>
@@ -8707,7 +8828,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="141">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18">
       <c r="A141" s="1" t="s">
         <v>469</v>
       </c>
@@ -8733,7 +8854,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="142">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18">
       <c r="A142" s="1" t="s">
         <v>469</v>
       </c>
@@ -8759,7 +8880,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="143">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18">
       <c r="A143" s="1" t="s">
         <v>469</v>
       </c>
@@ -8785,7 +8906,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="144">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18">
       <c r="A144" s="1" t="s">
         <v>469</v>
       </c>
@@ -8811,7 +8932,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="145">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18">
       <c r="A145" s="1" t="s">
         <v>469</v>
       </c>
@@ -8837,7 +8958,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="146">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18">
       <c r="A146" s="1" t="s">
         <v>487</v>
       </c>
@@ -8863,7 +8984,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="147">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18">
       <c r="A147" s="1" t="s">
         <v>487</v>
       </c>
@@ -8889,7 +9010,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="148">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18">
       <c r="A148" s="1" t="s">
         <v>487</v>
       </c>
@@ -8915,7 +9036,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="149">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18">
       <c r="A149" s="1" t="s">
         <v>487</v>
       </c>
@@ -8941,7 +9062,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="150">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18">
       <c r="A150" s="1" t="s">
         <v>487</v>
       </c>
@@ -8967,7 +9088,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="151">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18">
       <c r="A151" s="1" t="s">
         <v>487</v>
       </c>
@@ -8993,7 +9114,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="152">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18">
       <c r="A152" s="1" t="s">
         <v>487</v>
       </c>
@@ -9019,7 +9140,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="153">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18">
       <c r="A153" s="1" t="s">
         <v>504</v>
       </c>
@@ -9045,7 +9166,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="154">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18">
       <c r="A154" s="1" t="s">
         <v>509</v>
       </c>
@@ -9071,7 +9192,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="155">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18">
       <c r="A155" s="1" t="s">
         <v>509</v>
       </c>
@@ -9097,7 +9218,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="156">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18">
       <c r="A156" s="1" t="s">
         <v>517</v>
       </c>
@@ -9123,7 +9244,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="157">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18">
       <c r="A157" s="1" t="s">
         <v>522</v>
       </c>
@@ -9149,7 +9270,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="158">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18">
       <c r="A158" s="1" t="s">
         <v>522</v>
       </c>
@@ -9175,7 +9296,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="159">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18">
       <c r="A159" s="1" t="s">
         <v>522</v>
       </c>
@@ -9201,7 +9322,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="160">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18">
       <c r="A160" s="1" t="s">
         <v>522</v>
       </c>
@@ -9227,7 +9348,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="161">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18">
       <c r="A161" s="1" t="s">
         <v>522</v>
       </c>
@@ -9253,7 +9374,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="162">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18">
       <c r="A162" s="1" t="s">
         <v>522</v>
       </c>
@@ -9279,7 +9400,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="163">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18">
       <c r="A163" s="1" t="s">
         <v>537</v>
       </c>
@@ -9305,7 +9426,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="164">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18">
       <c r="A164" s="1" t="s">
         <v>537</v>
       </c>
@@ -9331,7 +9452,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="165">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18">
       <c r="A165" s="1" t="s">
         <v>537</v>
       </c>
@@ -9357,7 +9478,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="166">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18">
       <c r="A166" s="1" t="s">
         <v>537</v>
       </c>
@@ -9383,7 +9504,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="167">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18">
       <c r="A167" s="1" t="s">
         <v>537</v>
       </c>
@@ -9409,7 +9530,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="168">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18">
       <c r="A168" s="1" t="s">
         <v>537</v>
       </c>
@@ -9435,7 +9556,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="169">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18">
       <c r="A169" s="1" t="s">
         <v>537</v>
       </c>
@@ -9461,7 +9582,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="170">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18">
       <c r="A170" s="1" t="s">
         <v>537</v>
       </c>
@@ -9487,7 +9608,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="171">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18">
       <c r="A171" s="1" t="s">
         <v>557</v>
       </c>
@@ -9513,7 +9634,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="172">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18">
       <c r="A172" s="1" t="s">
         <v>562</v>
       </c>
@@ -9539,7 +9660,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="173">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18">
       <c r="A173" s="1" t="s">
         <v>562</v>
       </c>
@@ -9565,7 +9686,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="174">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18">
       <c r="A174" s="1" t="s">
         <v>568</v>
       </c>
@@ -9591,7 +9712,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="175">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18">
       <c r="A175" s="1" t="s">
         <v>568</v>
       </c>
@@ -9617,7 +9738,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="176">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18">
       <c r="A176" s="1" t="s">
         <v>575</v>
       </c>
@@ -9643,7 +9764,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="177">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18">
       <c r="A177" s="1" t="s">
         <v>575</v>
       </c>
@@ -9669,7 +9790,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="178">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18">
       <c r="A178" s="1" t="s">
         <v>580</v>
       </c>
@@ -9695,7 +9816,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="179">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18">
       <c r="A179" s="1" t="s">
         <v>585</v>
       </c>
@@ -9721,7 +9842,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="180">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18">
       <c r="A180" s="1" t="s">
         <v>585</v>
       </c>
@@ -9747,7 +9868,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="181">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18">
       <c r="A181" s="1" t="s">
         <v>592</v>
       </c>
@@ -9773,7 +9894,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="182">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18">
       <c r="A182" s="1" t="s">
         <v>597</v>
       </c>
@@ -9799,7 +9920,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="183">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18">
       <c r="A183" s="1" t="s">
         <v>602</v>
       </c>
@@ -9825,7 +9946,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="184">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18">
       <c r="A184" s="1" t="s">
         <v>607</v>
       </c>
@@ -9851,7 +9972,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="185">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18">
       <c r="A185" s="1" t="s">
         <v>607</v>
       </c>
@@ -9877,7 +9998,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="186">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18">
       <c r="A186" s="1" t="s">
         <v>607</v>
       </c>
@@ -9903,7 +10024,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="187">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18">
       <c r="A187" s="1" t="s">
         <v>607</v>
       </c>
@@ -9929,7 +10050,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="188">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18">
       <c r="A188" s="1" t="s">
         <v>618</v>
       </c>
@@ -9955,7 +10076,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="189">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18">
       <c r="A189" s="1" t="s">
         <v>623</v>
       </c>
@@ -9981,7 +10102,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="190">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18">
       <c r="A190" s="1" t="s">
         <v>628</v>
       </c>
@@ -10007,7 +10128,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="191">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18">
       <c r="A191" s="1" t="s">
         <v>633</v>
       </c>
@@ -10033,7 +10154,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="192">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18">
       <c r="A192" s="1" t="s">
         <v>633</v>
       </c>
@@ -10059,7 +10180,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="193">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18">
       <c r="A193" s="1" t="s">
         <v>640</v>
       </c>
@@ -10085,7 +10206,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="194">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18">
       <c r="A194" s="1" t="s">
         <v>640</v>
       </c>
@@ -10111,7 +10232,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="195">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18">
       <c r="A195" s="1" t="s">
         <v>640</v>
       </c>
@@ -10137,7 +10258,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="196">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18">
       <c r="A196" s="1" t="s">
         <v>640</v>
       </c>
@@ -10163,7 +10284,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="197">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18">
       <c r="A197" s="1" t="s">
         <v>640</v>
       </c>
@@ -10189,7 +10310,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="198">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18">
       <c r="A198" s="1" t="s">
         <v>640</v>
       </c>
@@ -10215,7 +10336,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="199">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18">
       <c r="A199" s="1" t="s">
         <v>640</v>
       </c>
@@ -10241,7 +10362,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="200">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18">
       <c r="A200" s="1" t="s">
         <v>658</v>
       </c>
@@ -10267,7 +10388,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="201">
+    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18">
       <c r="A201" s="1" t="s">
         <v>663</v>
       </c>
@@ -10294,49 +10415,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="C4"/>
-    <hyperlink r:id="rId2" ref="C6"/>
-    <hyperlink r:id="rId3" ref="C7"/>
-    <hyperlink r:id="rId4" ref="C8"/>
-    <hyperlink r:id="rId5" ref="C22"/>
-    <hyperlink r:id="rId6" ref="C29"/>
-    <hyperlink r:id="rId7" ref="C37"/>
-    <hyperlink r:id="rId8" ref="C38"/>
-    <hyperlink r:id="rId9" ref="C39"/>
-    <hyperlink r:id="rId10" ref="C41"/>
-    <hyperlink r:id="rId11" ref="C47"/>
-    <hyperlink r:id="rId12" ref="C57"/>
-    <hyperlink r:id="rId13" ref="C58"/>
-    <hyperlink r:id="rId14" ref="C59"/>
-    <hyperlink r:id="rId15" ref="C60"/>
-    <hyperlink r:id="rId16" ref="C108"/>
-    <hyperlink r:id="rId17" ref="C112"/>
-    <hyperlink r:id="rId18" ref="C113"/>
-    <hyperlink r:id="rId19" ref="C122"/>
-    <hyperlink r:id="rId20" ref="C123"/>
-    <hyperlink r:id="rId21" ref="C124"/>
-    <hyperlink r:id="rId22" ref="C125"/>
-    <hyperlink r:id="rId23" ref="C146"/>
-    <hyperlink r:id="rId24" ref="C147"/>
-    <hyperlink r:id="rId25" ref="C148"/>
-    <hyperlink r:id="rId26" ref="C149"/>
-    <hyperlink r:id="rId27" ref="C150"/>
-    <hyperlink r:id="rId28" ref="C151"/>
-    <hyperlink r:id="rId29" ref="C152"/>
-    <hyperlink r:id="rId30" ref="C157"/>
-    <hyperlink r:id="rId31" ref="C158"/>
-    <hyperlink r:id="rId32" ref="C159"/>
-    <hyperlink r:id="rId33" ref="C160"/>
-    <hyperlink r:id="rId34" ref="C161"/>
-    <hyperlink r:id="rId35" ref="C162"/>
-    <hyperlink r:id="rId36" ref="C181"/>
-    <hyperlink r:id="rId37" ref="C182"/>
-    <hyperlink r:id="rId38" ref="C184"/>
-    <hyperlink r:id="rId39" ref="C185"/>
-    <hyperlink r:id="rId40" ref="C186"/>
-    <hyperlink r:id="rId41" ref="C187"/>
-  </hyperlinks>
-  <drawing r:id="rId42"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>